<commit_message>
Add migration for supervision task fields and implement tests for graduation system functionality
- Created migration to add 'is_late' and 'submitted_at' fields to SupervisionTask model.
- Updated GraduationProject status choices in migration.
- Implemented comprehensive test cases for graduation system including:
  - Authorization checks for admin topic approval.
  - Status updates on topic resubmission.
  - Late task submission handling.
  - Academic grades import validation.
  - Council score finalization requirements.
  - Supervisor scoring restrictions.
  - Academic deferral request flow.
  - Defense schedule conflict detection.
  - Admin override for allocation quota.
  - Access restrictions for students on council minutes and final grades export.
</commit_message>
<xml_diff>
--- a/Bao_Cao_Ket_Qua_Kiem_Thu_Smart_FYP.xlsx
+++ b/Bao_Cao_Ket_Qua_Kiem_Thu_Smart_FYP.xlsx
@@ -9,7 +9,7 @@
   <sheets>
     <sheet name="Tổng Quan &amp; Thống Kê" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Chi Tiết Test Cases" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Toàn Bộ Test Suite (176 Tests)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Toàn Bộ Test Suite (186 Tests)" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="12">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -92,8 +92,24 @@
       <color rgb="000F5132"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="002E7D32"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00C62828"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -130,8 +146,20 @@
         <bgColor rgb="00F9FAFB"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8F5E9"/>
+        <bgColor rgb="00E8F5E9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEBEE"/>
+        <bgColor rgb="00FFEBEE"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -167,11 +195,85 @@
         <color rgb="001F497D"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D3D3D3"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D3D3D3"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D3D3D3"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D3D3D3"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D3D3D3"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D3D3D3"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00D3D3D3"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D3D3D3"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00D3D3D3"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00DDDDDD"/>
+      </left>
+      <right style="thin">
+        <color rgb="00DDDDDD"/>
+      </right>
+      <top style="thin">
+        <color rgb="00DDDDDD"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00DDDDDD"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -219,6 +321,23 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -619,7 +738,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>07/10/2026 12:05:00</t>
+          <t>10/10/2026 10:56:02</t>
         </is>
       </c>
     </row>
@@ -643,7 +762,7 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>11 Test Cases (100% PASS)</t>
+          <t>21 Test Cases (100% PASS - TC-001..007, TC_031..033, TC_039, TC-029..038)</t>
         </is>
       </c>
     </row>
@@ -655,7 +774,7 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>176 Tests (175 PASS, 1 Skipped, 0 Fail)</t>
+          <t>186 Tests (185 PASS, 1 Skipped, 0 Fail)</t>
         </is>
       </c>
     </row>
@@ -685,37 +804,37 @@
 11</t>
         </is>
       </c>
-      <c r="C12" s="7" t="n"/>
+      <c r="C12" s="20" t="n"/>
       <c r="D12" s="8" t="inlineStr">
         <is>
           <t>SỐ TC ĐẠT (PASS)
 11 (100%)</t>
         </is>
       </c>
-      <c r="E12" s="7" t="n"/>
+      <c r="E12" s="20" t="n"/>
       <c r="F12" s="9" t="inlineStr">
         <is>
           <t>SỐ TC LỖI (FAIL)
 0 (0%)</t>
         </is>
       </c>
-      <c r="G12" s="7" t="n"/>
+      <c r="G12" s="20" t="n"/>
     </row>
     <row r="13">
-      <c r="B13" s="7" t="n"/>
-      <c r="C13" s="7" t="n"/>
-      <c r="D13" s="7" t="n"/>
-      <c r="E13" s="7" t="n"/>
-      <c r="F13" s="7" t="n"/>
-      <c r="G13" s="7" t="n"/>
+      <c r="B13" s="21" t="n"/>
+      <c r="C13" s="22" t="n"/>
+      <c r="D13" s="21" t="n"/>
+      <c r="E13" s="22" t="n"/>
+      <c r="F13" s="21" t="n"/>
+      <c r="G13" s="22" t="n"/>
     </row>
     <row r="14">
-      <c r="B14" s="7" t="n"/>
-      <c r="C14" s="7" t="n"/>
-      <c r="D14" s="7" t="n"/>
-      <c r="E14" s="7" t="n"/>
-      <c r="F14" s="7" t="n"/>
-      <c r="G14" s="7" t="n"/>
+      <c r="B14" s="23" t="n"/>
+      <c r="C14" s="24" t="n"/>
+      <c r="D14" s="23" t="n"/>
+      <c r="E14" s="24" t="n"/>
+      <c r="F14" s="23" t="n"/>
+      <c r="G14" s="24" t="n"/>
     </row>
     <row r="16">
       <c r="B16" s="5" t="inlineStr">
@@ -973,7 +1092,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K14"/>
+  <dimension ref="A1:K24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1670,6 +1789,574 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="25" t="n">
+        <v>12</v>
+      </c>
+      <c r="B15" s="25" t="inlineStr">
+        <is>
+          <t>TC-029</t>
+        </is>
+      </c>
+      <c r="C15" s="26" t="inlineStr">
+        <is>
+          <t>Module 1 / Auth &amp; Security</t>
+        </is>
+      </c>
+      <c r="D15" s="26" t="inlineStr">
+        <is>
+          <t>Security &amp; Permission</t>
+        </is>
+      </c>
+      <c r="E15" s="26" t="inlineStr">
+        <is>
+          <t>Sinh viên gọi API duyệt đề tài của Khoa (/app/graduation-project/admin-approve-topic/). Hệ thống phải chặn và trả về HTTP 403 Forbidden.</t>
+        </is>
+      </c>
+      <c r="F15" s="26" t="inlineStr">
+        <is>
+          <t>POST /app/graduation-project/admin-approve-topic/
+Payload: {"project_id": X, "decision": "APPROVED"}
+User: Sinh viên (user_type="student") hoặc GV không phải staff</t>
+        </is>
+      </c>
+      <c r="G15" s="26" t="inlineStr">
+        <is>
+          <t>HTTP 403 Forbidden; Chặn sinh viên và người dùng không có thẩm quyền duyệt đề tài của Khoa.</t>
+        </is>
+      </c>
+      <c r="H15" s="26" t="inlineStr">
+        <is>
+          <t>HTTP 403 Forbidden với message: "Sinh viên không có quyền phê duyệt đề tài (Chỉ dành cho Khoa/Ban quản trị).". Admin/Ban chủ nhiệm duyệt thành công TOPIC_APPROVED.</t>
+        </is>
+      </c>
+      <c r="I15" s="27" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="J15" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K15" s="26" t="inlineStr">
+        <is>
+          <t>Bổ sung kiểm tra phân quyền chặt chẽ trong AdminApproveTopicAPIView: nếu user_type == student hoặc không phải Admin/Staff lập tức trả về HTTP 403 Forbidden.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="25" t="n">
+        <v>13</v>
+      </c>
+      <c r="B16" s="25" t="inlineStr">
+        <is>
+          <t>TC-030</t>
+        </is>
+      </c>
+      <c r="C16" s="26" t="inlineStr">
+        <is>
+          <t>Module 3 / Luồng Đề tài</t>
+        </is>
+      </c>
+      <c r="D16" s="26" t="inlineStr">
+        <is>
+          <t>Workflow &amp; Transition</t>
+        </is>
+      </c>
+      <c r="E16" s="26" t="inlineStr">
+        <is>
+          <t>Sau khi bị Khoa Từ chối hoặc Yêu cầu sửa (Draft/Revision), GV/SV chỉnh sửa lại nội dung đề tài và Re-Submit -&gt; Chuyển trạng thái lại thành Pending Review (PENDING_REVIEW).</t>
+        </is>
+      </c>
+      <c r="F16" s="26" t="inlineStr">
+        <is>
+          <t>POST /app/graduation-project/re-submit/
+Payload: {"project_id": X, "topic_title_vi": "...", "description": "..."}
+User: Sinh viên hoặc GVHD</t>
+        </is>
+      </c>
+      <c r="G16" s="26" t="inlineStr">
+        <is>
+          <t>Cập nhật thông tin đề tài và chuyển trạng thái project.status thành PENDING_REVIEW; đồng bộ nhóm đồ án sang PENDING_REVIEW; gửi thông báo cho Khoa.</t>
+        </is>
+      </c>
+      <c r="H16" s="26" t="inlineStr">
+        <is>
+          <t>HTTP 200 OK; Project chuyển trạng thái về PENDING_REVIEW; nhóm đồ án đồng bộ tentative_topic và topic_status="PENDING_REVIEW".</t>
+        </is>
+      </c>
+      <c r="I16" s="27" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="J16" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K16" s="26" t="inlineStr">
+        <is>
+          <t>Bổ sung giá trị PENDING_REVIEW vào STATUS_CHOICES của GraduationProject; xây dựng TopicReSubmitAPIView tại /app/graduation-project/re-submit/ và cập nhật TopicDraftAPIView.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="25" t="n">
+        <v>14</v>
+      </c>
+      <c r="B17" s="25" t="inlineStr">
+        <is>
+          <t>TC-031</t>
+        </is>
+      </c>
+      <c r="C17" s="26" t="inlineStr">
+        <is>
+          <t>Module 4 / Luồng Task</t>
+        </is>
+      </c>
+      <c r="D17" s="26" t="inlineStr">
+        <is>
+          <t>Boundary &amp; Validation</t>
+        </is>
+      </c>
+      <c r="E17" s="26" t="inlineStr">
+        <is>
+          <t>SV nộp bài (Submit Task) quá deadline -&gt; Hệ thống tự động gắn flag is_late = True ("Late Submit") hoặc chặn nộp khi bật strict deadline.</t>
+        </is>
+      </c>
+      <c r="F17" s="26" t="inlineStr">
+        <is>
+          <t>POST /app/student/tasks/&lt;pk&gt;/submit-deliverable/
+Payload: deliverable_file, deliverable_url, student_notes, strict=true/false
+Task có due_date &lt; ngày hiện tại</t>
+        </is>
+      </c>
+      <c r="G17" s="26" t="inlineStr">
+        <is>
+          <t>Nộp quá hạn: task.is_late = True, ghi nhận submitted_at; thông báo tới GVHD kèm nhãn [Late Submit]. Nếu strict=True: trả về HTTP 400 Bad Request chặn nộp bài.</t>
+        </is>
+      </c>
+      <c r="H17" s="26" t="inlineStr">
+        <is>
+          <t>Nộp quá hạn ghi nhận is_late=True, submitted_at=timezone.now(); với strict=True trả về HTTP 400 error="deadline_exceeded" chi tiết.</t>
+        </is>
+      </c>
+      <c r="I17" s="27" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="J17" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K17" s="26" t="inlineStr">
+        <is>
+          <t>Thêm trường is_late và submitted_at vào model SupervisionTask, tạo migration 0012; cập nhật StudentTaskDeliverableSubmitAPIView và StudentMarkTaskCompletedAPIView.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="25" t="n">
+        <v>15</v>
+      </c>
+      <c r="B18" s="25" t="inlineStr">
+        <is>
+          <t>TC-032</t>
+        </is>
+      </c>
+      <c r="C18" s="26" t="inlineStr">
+        <is>
+          <t>Module 5 / Luồng ĐK Học vụ</t>
+        </is>
+      </c>
+      <c r="D18" s="26" t="inlineStr">
+        <is>
+          <t>Negative &amp; Validation</t>
+        </is>
+      </c>
+      <c r="E18" s="26" t="inlineStr">
+        <is>
+          <t>Import file điểm Excel (Giáo vụ) bị lỗi định dạng / header hoặc dữ liệu dòng không hợp lệ -&gt; Báo lỗi chi tiết dòng lỗi (row_errors kèm số dòng, trường lỗi, nội dung lỗi).</t>
+        </is>
+      </c>
+      <c r="F18" s="26" t="inlineStr">
+        <is>
+          <t>POST /app/academic/grades/import/
+File Excel/CSV: thiếu header bắt buộc (MSSV/CPA/Tín chỉ) hoặc dòng chứa CPA &gt; 4.0, tín chỉ âm, MSSV không tồn tại</t>
+        </is>
+      </c>
+      <c r="G18" s="26" t="inlineStr">
+        <is>
+          <t>Trả về HTTP 400 Bad Request; nếu sai header trả về missing_columns; nếu sai dòng dữ liệu trả về mảng row_errors chi tiết từng dòng, không crash 500.</t>
+        </is>
+      </c>
+      <c r="H18" s="26" t="inlineStr">
+        <is>
+          <t>HTTP 400 Bad Request với invalid_header kèm missing_columns; hoặc invalid_rows_data kèm row_errors liệt kê chính xác số dòng và trường vi phạm.</t>
+        </is>
+      </c>
+      <c r="I18" s="27" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="J18" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K18" s="26" t="inlineStr">
+        <is>
+          <t>Xây dựng AcademicGradesImportAPIView hỗ trợ .xlsx, .xls, .csv; chuẩn hóa header tiếng Việt không dấu; xác thực chặt chẽ CPA (0.0-4.0), tín chỉ, tín chỉ nợ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="25" t="n">
+        <v>16</v>
+      </c>
+      <c r="B19" s="25" t="inlineStr">
+        <is>
+          <t>TC-033</t>
+        </is>
+      </c>
+      <c r="C19" s="26" t="inlineStr">
+        <is>
+          <t>Module 6 / Hội đồng &amp; Chấm điểm</t>
+        </is>
+      </c>
+      <c r="D19" s="26" t="inlineStr">
+        <is>
+          <t>Logic &amp; Constraint</t>
+        </is>
+      </c>
+      <c r="E19" s="26" t="inlineStr">
+        <is>
+          <t>Tổng hợp và chốt điểm Hội đồng nhưng chỉ có 4/5 thành viên Hội đồng đã nhập điểm -&gt; Báo lỗi: "Bắt buộc 5/5 người chấm mới cho phép chốt".</t>
+        </is>
+      </c>
+      <c r="F19" s="26" t="inlineStr">
+        <is>
+          <t>POST /app/council/&lt;id&gt;/finalize-scores/
+(hoặc POST /app/council/scores/aggregate/)
+Điều kiện: Hội đồng 5 thành viên, mới có 4 phiếu điểm trong CouncilLiveScore</t>
+        </is>
+      </c>
+      <c r="G19" s="26" t="inlineStr">
+        <is>
+          <t>Hệ thống từ chối khóa điểm, trả về HTTP 400 Bad Request kèm thông báo: "Bắt buộc 5/5 người chấm mới cho phép chốt.". Chỉ cho phép chốt khi đủ 5/5 phiếu điểm.</t>
+        </is>
+      </c>
+      <c r="H19" s="26" t="inlineStr">
+        <is>
+          <t>Trả về HTTP 400 Bad Request với detail: "Báo lỗi: Bắt buộc 5/5 người chấm mới cho phép chốt." và error="incomplete_scoring"; khi đủ 5/5 thì khóa điểm thành công.</t>
+        </is>
+      </c>
+      <c r="I19" s="27" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="J19" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K19" s="26" t="inlineStr">
+        <is>
+          <t>Cập nhật CouncilToggleLockAPIView và xây dựng CouncilFinalizeScoresAPIView, kiểm tra CouncilLiveScore.objects.filter(project=p, council=c).count() &gt;= required_scorers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="25" t="n">
+        <v>17</v>
+      </c>
+      <c r="B20" s="25" t="inlineStr">
+        <is>
+          <t>TC-034</t>
+        </is>
+      </c>
+      <c r="C20" s="26" t="inlineStr">
+        <is>
+          <t>Module 6 / Hội đồng &amp; Chấm điểm</t>
+        </is>
+      </c>
+      <c r="D20" s="26" t="inlineStr">
+        <is>
+          <t>Security &amp; Conflict (COI)</t>
+        </is>
+      </c>
+      <c r="E20" s="26" t="inlineStr">
+        <is>
+          <t>GV hướng dẫn tìm cách chấm điểm cho chính SV của mình trong màn hình Hội đồng bảo vệ -&gt; Chặn và báo lỗi Validation 403 Forbidden.</t>
+        </is>
+      </c>
+      <c r="F20" s="26" t="inlineStr">
+        <is>
+          <t>POST /app/council/submit-score/
+User: GVHD của project
+Payload: project_id, score_presentation, score_content, score_qa, score_demo</t>
+        </is>
+      </c>
+      <c r="G20" s="26" t="inlineStr">
+        <is>
+          <t>Trả về HTTP 403 Forbidden với message: "Vi phạm quy chế: Giảng viên hướng dẫn không được phép chấm điểm Hội đồng cho chính sinh viên của mình.".</t>
+        </is>
+      </c>
+      <c r="H20" s="26" t="inlineStr">
+        <is>
+          <t>HTTP 403 Forbidden, chặn hoàn toàn GVHD chấm điểm SV của mình trong Hội đồng; chỉ thành viên độc lập mới được chấm.</t>
+        </is>
+      </c>
+      <c r="I20" s="27" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="J20" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K20" s="26" t="inlineStr">
+        <is>
+          <t>Trong CouncilSubmitScoreAPIView, kiểm tra chéo quan hệ GVHD: (council_member.supervisor == project.supervisor or project.supervisor.user == user) -&gt; trả về HTTP 403 Forbidden.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="25" t="n">
+        <v>18</v>
+      </c>
+      <c r="B21" s="25" t="inlineStr">
+        <is>
+          <t>TC-035</t>
+        </is>
+      </c>
+      <c r="C21" s="26" t="inlineStr">
+        <is>
+          <t>Module 5 / Luồng Bảo lưu</t>
+        </is>
+      </c>
+      <c r="D21" s="26" t="inlineStr">
+        <is>
+          <t>Positive &amp; Workflow</t>
+        </is>
+      </c>
+      <c r="E21" s="26" t="inlineStr">
+        <is>
+          <t>Sinh viên không đủ điều kiện học vụ hoặc gặp lý do bất khả kháng nộp đơn xin bảo lưu; Khoa phê duyệt đơn bảo lưu đồ án.</t>
+        </is>
+      </c>
+      <c r="F21" s="26" t="inlineStr">
+        <is>
+          <t>POST /app/student/deferral-request/
+POST /app/admin/deferral-request/&lt;id&gt;/review/ với decision="APPROVED"</t>
+        </is>
+      </c>
+      <c r="G21" s="26" t="inlineStr">
+        <is>
+          <t>Tạo ThesisDeferralRequest status=PENDING; Admin duyệt chuyển status=APPROVED, project.status chuyển thành DEFERRED.</t>
+        </is>
+      </c>
+      <c r="H21" s="26" t="inlineStr">
+        <is>
+          <t>Nộp đơn thành công HTTP 201 Created; Khoa duyệt thành công HTTP 200 OK, project chuyển trạng thái DEFERRED và xuất hiện trong danh sách bảo lưu.</t>
+        </is>
+      </c>
+      <c r="I21" s="27" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J21" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K21" s="26" t="inlineStr">
+        <is>
+          <t>Hoàn thiện toàn diện luồng ThesisDeferralRequest, StudentDeferralRequestAPIView, AdminReviewDeferralRequestAPIView, đồng bộ trạng thái đồ án DEFERRED.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="25" t="n">
+        <v>19</v>
+      </c>
+      <c r="B22" s="25" t="inlineStr">
+        <is>
+          <t>TC-036</t>
+        </is>
+      </c>
+      <c r="C22" s="26" t="inlineStr">
+        <is>
+          <t>Module 6 / Lịch Bảo vệ</t>
+        </is>
+      </c>
+      <c r="D22" s="26" t="inlineStr">
+        <is>
+          <t>Business Logic &amp; Conflict</t>
+        </is>
+      </c>
+      <c r="E22" s="26" t="inlineStr">
+        <is>
+          <t>Xếp lịch cho 1 GV phản biện (hoặc ủy viên, hoặc phòng bảo vệ) bị trùng giờ trong 2 Hội đồng khác nhau -&gt; Báo lỗi xung đột lịch (Conflict Schedule).</t>
+        </is>
+      </c>
+      <c r="F22" s="26" t="inlineStr">
+        <is>
+          <t>POST /app/council/schedule/
+Payload: council_id, session_date, session_time, defense_room
+Điều kiện: Thành viên/Reviewer đã có lịch ở Council khác cùng ngày và ca</t>
+        </is>
+      </c>
+      <c r="G22" s="26" t="inlineStr">
+        <is>
+          <t>Trả về HTTP 400 Bad Request; message thông báo "Báo lỗi xung đột lịch (Conflict Schedule)" và danh sách conflicts chi tiết.</t>
+        </is>
+      </c>
+      <c r="H22" s="26" t="inlineStr">
+        <is>
+          <t>HTTP 400 Bad Request với detail chứa "Conflict Schedule", error="conflict_schedule", mảng conflicts chứa tên GV/phòng và tên Hội đồng bị trùng.</t>
+        </is>
+      </c>
+      <c r="I22" s="27" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="J22" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K22" s="26" t="inlineStr">
+        <is>
+          <t>Trong CouncilScheduleDefenseAPIView, quét chéo all members, reviewers và phòng bảo vệ của other_councils cùng session_date và session_time; trả về xung đột nếu trùng.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="25" t="n">
+        <v>20</v>
+      </c>
+      <c r="B23" s="25" t="inlineStr">
+        <is>
+          <t>TC-037</t>
+        </is>
+      </c>
+      <c r="C23" s="26" t="inlineStr">
+        <is>
+          <t>Module 2 / Admin Phân công</t>
+        </is>
+      </c>
+      <c r="D23" s="26" t="inlineStr">
+        <is>
+          <t>Exception &amp; Quota Override</t>
+        </is>
+      </c>
+      <c r="E23" s="26" t="inlineStr">
+        <is>
+          <t>Tính năng Force Assign - Admin cố tình gán 1 SV cho GV đã đầy Slot -&gt; Cảnh báo nhưng vẫn cho phép lưu khi có cờ xác nhận (Override).</t>
+        </is>
+      </c>
+      <c r="F23" s="26" t="inlineStr">
+        <is>
+          <t>POST /app/allocation/override/
+Payload: allocation_id, supervisor_id, force=true/false
+Điều kiện: GV đã đủ chỉ tiêu max_quota</t>
+        </is>
+      </c>
+      <c r="G23" s="26" t="inlineStr">
+        <is>
+          <t>Khi chưa có force: trả về HTTP 400 Bad Request cảnh báo is_quota_exceeded: True và can_override: True. Khi có force=True: cho phép lưu HTTP 200 OK kèm warning.</t>
+        </is>
+      </c>
+      <c r="H23" s="26" t="inlineStr">
+        <is>
+          <t>Chưa force trả về HTTP 400 cảnh báo đầy slot; có force=True lưu thành công HTTP 200 OK, cập nhật GVHD mới và ghi nhận is_overridden=True.</t>
+        </is>
+      </c>
+      <c r="I23" s="27" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="J23" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K23" s="26" t="inlineStr">
+        <is>
+          <t>Cập nhật OverrideAllocationAPIView tính current_assigned so với max_quota; nếu đầy slot và force=False -&gt; trả về 400 với can_override=True; nếu force=True -&gt; cho phép override.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="25" t="n">
+        <v>21</v>
+      </c>
+      <c r="B24" s="25" t="inlineStr">
+        <is>
+          <t>TC-038</t>
+        </is>
+      </c>
+      <c r="C24" s="26" t="inlineStr">
+        <is>
+          <t>Module 6 / Security / Export</t>
+        </is>
+      </c>
+      <c r="D24" s="26" t="inlineStr">
+        <is>
+          <t>Security &amp; Authorization</t>
+        </is>
+      </c>
+      <c r="E24" s="26" t="inlineStr">
+        <is>
+          <t>Sinh viên truy cập vào link URL Export PDF Biên bản hoặc Bảng điểm tốt nghiệp (dành cho Khoa) -&gt; Phải chặn và trả Lỗi 403 Forbidden.</t>
+        </is>
+      </c>
+      <c r="F24" s="26" t="inlineStr">
+        <is>
+          <t>GET /app/council/&lt;id&gt;/export-minutes-pdf/
+GET /app/batch/&lt;id&gt;/export-final-grades-excel/
+User: Sinh viên (user_type="student")</t>
+        </is>
+      </c>
+      <c r="G24" s="26" t="inlineStr">
+        <is>
+          <t>Trả về HTTP 403 Forbidden với message: "Sinh viên không có quyền truy cập hoặc tải về Biên bản họp Hội đồng bảo vệ." / "Bảng điểm tốt nghiệp.". Chỉ Admin và GV mới được tải.</t>
+        </is>
+      </c>
+      <c r="H24" s="26" t="inlineStr">
+        <is>
+          <t>Sinh viên gọi GET bị chặn 100% với HTTP 403 Forbidden; Admin và GVHD gọi GET trả về HTTP 200 OK với file PDF/Excel chuẩn.</t>
+        </is>
+      </c>
+      <c r="I24" s="27" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="J24" s="28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K24" s="26" t="inlineStr">
+        <is>
+          <t>Bổ sung kiểm tra quyền trong CouncilMinutesPdfExportAPIView và BatchFinalGradesExcelExportAPIView: chặn tuyệt đối user_type == student bằng HTTP 403 Forbidden.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:K1"/>
@@ -1684,7 +2371,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1698,7 +2385,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>DANH SÁCH CÁC MODULE KIỂM THỬ TỰ ĐỘNG TOÀN HỆ THỐNG (176 TESTS)</t>
+          <t>DANH SÁCH CÁC MODULE KIỂM THỬ TỰ ĐỘNG TOÀN HỆ THỐNG (186 TESTS)</t>
         </is>
       </c>
     </row>
@@ -2015,26 +2702,54 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="inlineStr"/>
-      <c r="B14" s="15" t="inlineStr">
+      <c r="A14" s="25" t="n">
+        <v>11</v>
+      </c>
+      <c r="B14" s="26" t="inlineStr">
+        <is>
+          <t>app.tests.test_utc_tc029_to_tc038</t>
+        </is>
+      </c>
+      <c r="C14" s="25" t="n">
+        <v>10</v>
+      </c>
+      <c r="D14" s="28" t="inlineStr">
+        <is>
+          <t>10 PASS</t>
+        </is>
+      </c>
+      <c r="E14" s="25" t="inlineStr">
+        <is>
+          <t>0.38s</t>
+        </is>
+      </c>
+      <c r="F14" s="26" t="inlineStr">
+        <is>
+          <t>Bao gồm 10 Test Cases trọng điểm đợt mới: TC-029 đến TC-038</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr"/>
+      <c r="B15" s="15" t="inlineStr">
         <is>
           <t>TỔNG SỐ TEST TOÀN DỰ ÁN</t>
         </is>
       </c>
-      <c r="C14" s="16" t="n">
-        <v>176</v>
-      </c>
-      <c r="D14" s="14" t="inlineStr">
-        <is>
-          <t>175 PASS, 1 SKIP</t>
-        </is>
-      </c>
-      <c r="E14" s="16" t="inlineStr">
-        <is>
-          <t>5.59s</t>
-        </is>
-      </c>
-      <c r="F14" s="15" t="inlineStr">
+      <c r="C15" s="16" t="n">
+        <v>186</v>
+      </c>
+      <c r="D15" s="14" t="inlineStr">
+        <is>
+          <t>185 PASS, 1 SKIP</t>
+        </is>
+      </c>
+      <c r="E15" s="16" t="inlineStr">
+        <is>
+          <t>4.66s</t>
+        </is>
+      </c>
+      <c r="F15" s="15" t="inlineStr">
         <is>
           <t>100% SUCCESS RATE</t>
         </is>

</xml_diff>